<commit_message>
Trying to make comments more succinct
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/project_tracker_matchmaking_leaderboard.xlsx
+++ b/Iteration_2/Echo_Review/Echo/project_tracker_matchmaking_leaderboard.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345C0D5B-3956-4E92-A84C-14C4ED877C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1852A5D3-2D31-41FB-B570-3C70AFB54719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,7 +79,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    According to the actual start dates, Student 3 started late, beginning on the day of the deadline. While the workload was less than expected and the deadline was met, this could be a sign of procrastination or rushed inadequate work and  should be addressed to see if the late start was the cause of student 3’s work ethic, a mistake in forgetting to adjust the expected start dates (as they don’t match the expected duration in days), or external matters.</t>
+    According to the actual start dates, Student 3 started late, beginning on the day of the deadline. While the workload was less than expected and the deadline was met, this discrepancy should be addressed. If it was caused by forgetting to change the estimated start date (as the estimated start and end don’t match the estimated duration), then adjust the estimated start date to match actual start and estimated duration</t>
       </text>
     </comment>
     <comment ref="L9" authorId="4" shapeId="0" xr:uid="{1E40B37D-EE5E-4ABA-94C6-CD6810B21150}">
@@ -1613,7 +1613,7 @@
     <text>Student 3’s estimated start and finish date for their tasks doesn’t match the estimated duration in days. This should be changed so that the expected start and finish dates should better align with the estimated duration</text>
   </threadedComment>
   <threadedComment ref="H9" dT="2024-11-14T04:12:11.23" personId="{00000000-0000-0000-0000-000000000000}" id="{9717BCA1-AFAA-4CBA-9F0B-F41FAF647A1C}">
-    <text>According to the actual start dates, Student 3 started late, beginning on the day of the deadline. While the workload was less than expected and the deadline was met, this could be a sign of procrastination or rushed inadequate work and  should be addressed to see if the late start was the cause of student 3’s work ethic, a mistake in forgetting to adjust the expected start dates (as they don’t match the expected duration in days), or external matters.</text>
+    <text>According to the actual start dates, Student 3 started late, beginning on the day of the deadline. While the workload was less than expected and the deadline was met, this discrepancy should be addressed. If it was caused by forgetting to change the estimated start date (as the estimated start and end don’t match the estimated duration), then adjust the estimated start date to match actual start and estimated duration</text>
   </threadedComment>
   <threadedComment ref="L9" dT="2024-11-13T02:22:05.30" personId="{00000000-0000-0000-0000-000000000000}" id="{1E40B37D-EE5E-4ABA-94C6-CD6810B21150}">
     <text>Student 3’s tasks have no notes. It would be helpful to have them to describe the tasks that student 3 has done and better track the overall state and progress of the project</text>

</xml_diff>